<commit_message>
Fix: Allow row/column resizing in WC Upload Template
Users could not resize rows or columns in the protected template,
making it challenging to type and review entries. Updated sheet
protection to permit formatCells, formatRows, and formatColumns
while still protecting header structure. Regenerated the template.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/bpc_upload_template/BPC1_WC_Upload_Template.xlsx
+++ b/bpc_upload_template/BPC1_WC_Upload_Template.xlsx
@@ -507,7 +507,7 @@
     <row r="1" ht="35" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>BPC2 Wins &amp; Challenges Upload Template</t>
+          <t>BPC1 Wins &amp; Challenges Upload Template</t>
         </is>
       </c>
     </row>
@@ -849,7 +849,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
@@ -1017,7 +1017,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>
@@ -1185,7 +1185,7 @@
       </c>
     </row>
   </sheetData>
-  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
+  <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="0" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="0" sort="1"/>
   <mergeCells count="1">
     <mergeCell ref="A1:B1"/>
   </mergeCells>

</xml_diff>